<commit_message>
11 03 2026 commit
</commit_message>
<xml_diff>
--- a/test-pdfs/rnd_7s.xlsx
+++ b/test-pdfs/rnd_7s.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects Java\QrCodeGenerator\test-pdfs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3B6A9E-2BC0-4F0B-A11F-408EB19A6AE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A08AB9B9-5133-40F0-8784-FCAC0A799DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -391,9 +391,6 @@
     <t>ГОСТ 7473-2010</t>
   </si>
   <si>
-    <t>В30</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="12"/>
@@ -538,6 +535,9 @@
       </rPr>
       <t>Э.И.Абливапов</t>
     </r>
+  </si>
+  <si>
+    <t>В20</t>
   </si>
 </sst>
 </file>
@@ -924,80 +924,80 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1406,37 +1406,37 @@
       <c r="C9" s="1"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="48" t="s">
-        <v>39</v>
+      <c r="A10" s="24" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="29"/>
-      <c r="C12" s="29"/>
-      <c r="D12" s="29"/>
-      <c r="E12" s="29"/>
-      <c r="F12" s="29"/>
-      <c r="G12" s="29"/>
-      <c r="H12" s="29"/>
-      <c r="I12" s="29"/>
-      <c r="J12" s="29"/>
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="25"/>
+      <c r="I12" s="25"/>
+      <c r="J12" s="25"/>
     </row>
     <row r="13" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="33"/>
-      <c r="C13" s="33"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="34"/>
-      <c r="I13" s="34"/>
-      <c r="J13" s="34"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="30"/>
+      <c r="J13" s="30"/>
     </row>
     <row r="14" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A14" s="5"/>
@@ -1493,30 +1493,30 @@
       <c r="J17" s="13"/>
     </row>
     <row r="18" spans="1:10" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="36" t="s">
-        <v>32</v>
-      </c>
-      <c r="B18" s="36"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="37"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="37"/>
-      <c r="I18" s="37"/>
-      <c r="J18" s="37"/>
+      <c r="A18" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="32"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="33"/>
+      <c r="J18" s="33"/>
     </row>
     <row r="19" spans="1:10" s="11" customFormat="1" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="35" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="35"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="35"/>
+      <c r="A19" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="31"/>
       <c r="G19" s="12" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="H19" s="12" t="s">
         <v>29</v>
@@ -1552,7 +1552,7 @@
     </row>
     <row r="22" spans="1:10" s="11" customFormat="1" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
@@ -1566,7 +1566,7 @@
     </row>
     <row r="23" spans="1:10" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A23" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
@@ -1729,8 +1729,8 @@
       <c r="B35" s="18"/>
       <c r="C35" s="18"/>
       <c r="D35" s="21" t="str">
-        <f>IF(G19="В20",F37,F36)</f>
-        <v>R = 1,5 * 10^(-2) * V - 2,5 * 10; Мпа</v>
+        <f>IF(OR(G19="В20", G19="B20"),F37,F36)</f>
+        <v>R = 1,45 * 10^(-2) * V - 2,5 * 10; Мпа</v>
       </c>
       <c r="E35" s="9"/>
       <c r="F35" s="8"/>
@@ -1764,7 +1764,7 @@
       <c r="D37" s="8"/>
       <c r="E37" s="8"/>
       <c r="F37" s="22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G37" s="8"/>
       <c r="H37" s="8"/>
@@ -1808,237 +1808,237 @@
       <c r="B44" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C44" s="38" t="s">
+      <c r="C44" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="D44" s="39"/>
+      <c r="D44" s="35"/>
       <c r="E44" s="3" t="s">
         <v>8</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G44" s="38" t="s">
+      <c r="G44" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="H44" s="39"/>
+      <c r="H44" s="35"/>
     </row>
     <row r="45" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
       <c r="B45" s="4">
         <v>1</v>
       </c>
-      <c r="C45" s="46">
+      <c r="C45" s="42">
         <v>2</v>
       </c>
-      <c r="D45" s="47"/>
+      <c r="D45" s="43"/>
       <c r="E45" s="4">
         <v>3</v>
       </c>
       <c r="F45" s="4">
         <v>4</v>
       </c>
-      <c r="G45" s="46">
+      <c r="G45" s="42">
         <v>5</v>
       </c>
-      <c r="H45" s="47"/>
+      <c r="H45" s="43"/>
     </row>
     <row r="46" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="B46" s="30" t="s">
+      <c r="B46" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C46" s="24">
+      <c r="C46" s="44">
         <v>1</v>
       </c>
-      <c r="D46" s="25"/>
+      <c r="D46" s="45"/>
       <c r="E46" s="4">
-        <f ca="1">IF($G$19="В30",RANDBETWEEN(3750,3950),IF($G$19="В25",RANDBETWEEN(3450,3650),RANDBETWEEN(3100,3350)))</f>
-        <v>3921</v>
+        <f ca="1">IF($G$19="В30",RANDBETWEEN(3750,3950),IF($G$19="В25",RANDBETWEEN(3450,3650),IF($G$19="B30",RANDBETWEEN(3750,3950),IF($G$19="B25",RANDBETWEEN(3450,3650),RANDBETWEEN(3100,3350)))))</f>
+        <v>3102</v>
       </c>
       <c r="F46" s="20">
         <f ca="1">$C$57*POWER(10,-2)*E46-2.5*10</f>
-        <v>33.814999999999998</v>
-      </c>
-      <c r="G46" s="40">
+        <v>19.978999999999999</v>
+      </c>
+      <c r="G46" s="36">
         <f ca="1">AVERAGE(F46:F55)</f>
-        <v>32.775500000000001</v>
-      </c>
-      <c r="H46" s="41"/>
+        <v>21.589949999999995</v>
+      </c>
+      <c r="H46" s="37"/>
     </row>
     <row r="47" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="B47" s="31"/>
-      <c r="C47" s="24">
+      <c r="B47" s="27"/>
+      <c r="C47" s="44">
         <v>2</v>
       </c>
-      <c r="D47" s="25">
+      <c r="D47" s="45">
         <v>2</v>
       </c>
       <c r="E47" s="4">
-        <f t="shared" ref="E47:E55" ca="1" si="0">IF($G$19="В30",RANDBETWEEN(3750,3950),IF($G$19="В25",RANDBETWEEN(3450,3650),RANDBETWEEN(3100,3350)))</f>
-        <v>3784</v>
+        <f t="shared" ref="E47:E55" ca="1" si="0">IF($G$19="В30",RANDBETWEEN(3750,3950),IF($G$19="В25",RANDBETWEEN(3450,3650),IF($G$19="B30",RANDBETWEEN(3750,3950),IF($G$19="B25",RANDBETWEEN(3450,3650),RANDBETWEEN(3100,3350)))))</f>
+        <v>3165</v>
       </c>
       <c r="F47" s="20">
         <f ca="1">$C$57*POWER(10,-2)*E47-2.5*10</f>
-        <v>31.759999999999998</v>
-      </c>
-      <c r="G47" s="42"/>
-      <c r="H47" s="43"/>
+        <v>20.892499999999998</v>
+      </c>
+      <c r="G47" s="38"/>
+      <c r="H47" s="39"/>
     </row>
     <row r="48" spans="1:10" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="B48" s="31"/>
-      <c r="C48" s="24">
+      <c r="B48" s="27"/>
+      <c r="C48" s="44">
         <v>3</v>
       </c>
-      <c r="D48" s="25">
+      <c r="D48" s="45">
         <v>3</v>
       </c>
       <c r="E48" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3836</v>
+        <v>3132</v>
       </c>
       <c r="F48" s="20">
         <f ca="1">$C$57*POWER(10,-2)*E48-2.5*10</f>
-        <v>32.54</v>
-      </c>
-      <c r="G48" s="42"/>
-      <c r="H48" s="43"/>
+        <v>20.413999999999994</v>
+      </c>
+      <c r="G48" s="38"/>
+      <c r="H48" s="39"/>
     </row>
     <row r="49" spans="2:8" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="B49" s="31"/>
-      <c r="C49" s="24">
+      <c r="B49" s="27"/>
+      <c r="C49" s="44">
         <v>4</v>
       </c>
-      <c r="D49" s="25">
+      <c r="D49" s="45">
         <v>4</v>
       </c>
       <c r="E49" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3892</v>
+        <v>3297</v>
       </c>
       <c r="F49" s="20">
         <f t="shared" ref="F49:F55" ca="1" si="1">$C$57*POWER(10,-2)*E49-2.5*10</f>
-        <v>33.379999999999995</v>
-      </c>
-      <c r="G49" s="42"/>
-      <c r="H49" s="43"/>
+        <v>22.8065</v>
+      </c>
+      <c r="G49" s="38"/>
+      <c r="H49" s="39"/>
     </row>
     <row r="50" spans="2:8" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="B50" s="31"/>
-      <c r="C50" s="24">
+      <c r="B50" s="27"/>
+      <c r="C50" s="44">
         <v>5</v>
       </c>
-      <c r="D50" s="25">
+      <c r="D50" s="45">
         <v>5</v>
       </c>
       <c r="E50" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3934</v>
+        <v>3180</v>
       </c>
       <c r="F50" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>34.01</v>
-      </c>
-      <c r="G50" s="42"/>
-      <c r="H50" s="43"/>
+        <v>21.11</v>
+      </c>
+      <c r="G50" s="38"/>
+      <c r="H50" s="39"/>
     </row>
     <row r="51" spans="2:8" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="B51" s="31"/>
-      <c r="C51" s="24">
+      <c r="B51" s="27"/>
+      <c r="C51" s="44">
         <v>6</v>
       </c>
-      <c r="D51" s="25">
+      <c r="D51" s="45">
         <v>6</v>
       </c>
       <c r="E51" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3832</v>
+        <v>3343</v>
       </c>
       <c r="F51" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>32.479999999999997</v>
-      </c>
-      <c r="G51" s="42"/>
-      <c r="H51" s="43"/>
+        <v>23.473499999999994</v>
+      </c>
+      <c r="G51" s="38"/>
+      <c r="H51" s="39"/>
     </row>
     <row r="52" spans="2:8" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="B52" s="31"/>
-      <c r="C52" s="24">
+      <c r="B52" s="27"/>
+      <c r="C52" s="44">
         <v>7</v>
       </c>
-      <c r="D52" s="25">
+      <c r="D52" s="45">
         <v>7</v>
       </c>
       <c r="E52" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3942</v>
+        <v>3244</v>
       </c>
       <c r="F52" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>34.129999999999995</v>
-      </c>
-      <c r="G52" s="42"/>
-      <c r="H52" s="43"/>
+        <v>22.037999999999997</v>
+      </c>
+      <c r="G52" s="38"/>
+      <c r="H52" s="39"/>
     </row>
     <row r="53" spans="2:8" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="B53" s="31"/>
-      <c r="C53" s="24">
+      <c r="B53" s="27"/>
+      <c r="C53" s="44">
         <v>8</v>
       </c>
-      <c r="D53" s="25">
+      <c r="D53" s="45">
         <v>8</v>
       </c>
       <c r="E53" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3841</v>
+        <v>3202</v>
       </c>
       <c r="F53" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>32.614999999999995</v>
-      </c>
-      <c r="G53" s="42"/>
-      <c r="H53" s="43"/>
+        <v>21.428999999999995</v>
+      </c>
+      <c r="G53" s="38"/>
+      <c r="H53" s="39"/>
     </row>
     <row r="54" spans="2:8" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="B54" s="31"/>
-      <c r="C54" s="24">
+      <c r="B54" s="27"/>
+      <c r="C54" s="44">
         <v>9</v>
       </c>
-      <c r="D54" s="25">
+      <c r="D54" s="45">
         <v>9</v>
       </c>
       <c r="E54" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3762</v>
+        <v>3321</v>
       </c>
       <c r="F54" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>31.43</v>
-      </c>
-      <c r="G54" s="42"/>
-      <c r="H54" s="43"/>
+        <v>23.154499999999999</v>
+      </c>
+      <c r="G54" s="38"/>
+      <c r="H54" s="39"/>
     </row>
     <row r="55" spans="2:8" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="B55" s="32"/>
-      <c r="C55" s="26">
+      <c r="B55" s="28"/>
+      <c r="C55" s="47">
         <v>10</v>
       </c>
-      <c r="D55" s="27">
+      <c r="D55" s="48">
         <v>10</v>
       </c>
       <c r="E55" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3773</v>
+        <v>3145</v>
       </c>
       <c r="F55" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>31.594999999999999</v>
-      </c>
-      <c r="G55" s="44"/>
-      <c r="H55" s="45"/>
+        <v>20.602499999999999</v>
+      </c>
+      <c r="G55" s="40"/>
+      <c r="H55" s="41"/>
     </row>
     <row r="57" spans="2:8" x14ac:dyDescent="0.2">
       <c r="C57" s="23">
-        <f>IF(G19="В20",1.45,1.5)</f>
-        <v>1.5</v>
+        <f>IF(OR(G19="В20", G19="B20"),1.45,1.5)</f>
+        <v>1.45</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
@@ -2046,12 +2046,12 @@
     </row>
     <row r="76" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A76" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="77" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F77" t="s">
         <v>13</v>
@@ -2063,57 +2063,64 @@
       </c>
     </row>
     <row r="82" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="28"/>
-      <c r="B82" s="28"/>
-      <c r="C82" s="28"/>
-      <c r="D82" s="28"/>
-      <c r="E82" s="28"/>
-      <c r="F82" s="28"/>
-      <c r="G82" s="28"/>
-      <c r="H82" s="28"/>
-      <c r="I82" s="28"/>
-      <c r="J82" s="28"/>
+      <c r="A82" s="46"/>
+      <c r="B82" s="46"/>
+      <c r="C82" s="46"/>
+      <c r="D82" s="46"/>
+      <c r="E82" s="46"/>
+      <c r="F82" s="46"/>
+      <c r="G82" s="46"/>
+      <c r="H82" s="46"/>
+      <c r="I82" s="46"/>
+      <c r="J82" s="46"/>
     </row>
     <row r="83" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="28"/>
-      <c r="B83" s="28"/>
-      <c r="C83" s="28"/>
-      <c r="D83" s="28"/>
-      <c r="E83" s="28"/>
-      <c r="F83" s="28"/>
-      <c r="G83" s="28"/>
-      <c r="H83" s="28"/>
-      <c r="I83" s="28"/>
-      <c r="J83" s="28"/>
+      <c r="A83" s="46"/>
+      <c r="B83" s="46"/>
+      <c r="C83" s="46"/>
+      <c r="D83" s="46"/>
+      <c r="E83" s="46"/>
+      <c r="F83" s="46"/>
+      <c r="G83" s="46"/>
+      <c r="H83" s="46"/>
+      <c r="I83" s="46"/>
+      <c r="J83" s="46"/>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A84" s="28" t="s">
-        <v>36</v>
-      </c>
-      <c r="B84" s="28"/>
-      <c r="C84" s="28"/>
-      <c r="D84" s="28"/>
-      <c r="E84" s="28"/>
-      <c r="F84" s="28"/>
-      <c r="G84" s="28"/>
-      <c r="H84" s="28"/>
-      <c r="I84" s="28"/>
-      <c r="J84" s="28"/>
+      <c r="A84" s="46" t="s">
+        <v>35</v>
+      </c>
+      <c r="B84" s="46"/>
+      <c r="C84" s="46"/>
+      <c r="D84" s="46"/>
+      <c r="E84" s="46"/>
+      <c r="F84" s="46"/>
+      <c r="G84" s="46"/>
+      <c r="H84" s="46"/>
+      <c r="I84" s="46"/>
+      <c r="J84" s="46"/>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A85" s="28"/>
-      <c r="B85" s="28"/>
-      <c r="C85" s="28"/>
-      <c r="D85" s="28"/>
-      <c r="E85" s="28"/>
-      <c r="F85" s="28"/>
-      <c r="G85" s="28"/>
-      <c r="H85" s="28"/>
-      <c r="I85" s="28"/>
-      <c r="J85" s="28"/>
+      <c r="A85" s="46"/>
+      <c r="B85" s="46"/>
+      <c r="C85" s="46"/>
+      <c r="D85" s="46"/>
+      <c r="E85" s="46"/>
+      <c r="F85" s="46"/>
+      <c r="G85" s="46"/>
+      <c r="H85" s="46"/>
+      <c r="I85" s="46"/>
+      <c r="J85" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A82:J83"/>
+    <mergeCell ref="A84:J85"/>
+    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="C52:D52"/>
+    <mergeCell ref="C53:D53"/>
+    <mergeCell ref="C54:D54"/>
+    <mergeCell ref="C55:D55"/>
     <mergeCell ref="A12:J12"/>
     <mergeCell ref="B46:B55"/>
     <mergeCell ref="A13:J13"/>
@@ -2130,13 +2137,6 @@
     <mergeCell ref="C48:D48"/>
     <mergeCell ref="C49:D49"/>
     <mergeCell ref="C50:D50"/>
-    <mergeCell ref="C51:D51"/>
-    <mergeCell ref="C52:D52"/>
-    <mergeCell ref="C53:D53"/>
-    <mergeCell ref="C54:D54"/>
-    <mergeCell ref="C55:D55"/>
-    <mergeCell ref="A82:J83"/>
-    <mergeCell ref="A84:J85"/>
   </mergeCells>
   <pageMargins left="0.43307086614173229" right="0.23622047244094491" top="0.51181102362204722" bottom="0.51181102362204722" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
15 08 2026 commit
</commit_message>
<xml_diff>
--- a/test-pdfs/rnd_7s.xlsx
+++ b/test-pdfs/rnd_7s.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="124226"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <workbookPr codeName="ЭтаКнига" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects Java\QrCodeGenerator\test-pdfs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A08AB9B9-5133-40F0-8784-FCAC0A799DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3120404A-9A80-45DD-966C-7CCD85DAE2B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -851,7 +851,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -998,6 +998,9 @@
     </xf>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1371,6 +1374,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr codeName="Лист1"/>
   <dimension ref="A7:J85"/>
   <sheetFormatPr defaultColWidth="9.33203125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1492,19 +1496,19 @@
       <c r="I17" s="12"/>
       <c r="J17" s="13"/>
     </row>
-    <row r="18" spans="1:10" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="32" t="s">
         <v>31</v>
       </c>
       <c r="B18" s="32"/>
       <c r="C18" s="32"/>
       <c r="D18" s="33"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="33"/>
-      <c r="G18" s="33"/>
-      <c r="H18" s="33"/>
-      <c r="I18" s="33"/>
-      <c r="J18" s="33"/>
+      <c r="E18" s="49"/>
+      <c r="F18" s="49"/>
+      <c r="G18" s="49"/>
+      <c r="H18" s="49"/>
+      <c r="I18" s="49"/>
+      <c r="J18" s="49"/>
     </row>
     <row r="19" spans="1:10" s="11" customFormat="1" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="31" t="s">
@@ -1852,15 +1856,15 @@
       <c r="D46" s="45"/>
       <c r="E46" s="4">
         <f ca="1">IF($G$19="В30",RANDBETWEEN(3750,3950),IF($G$19="В25",RANDBETWEEN(3450,3650),IF($G$19="B30",RANDBETWEEN(3750,3950),IF($G$19="B25",RANDBETWEEN(3450,3650),RANDBETWEEN(3100,3350)))))</f>
-        <v>3102</v>
+        <v>3319</v>
       </c>
       <c r="F46" s="20">
         <f ca="1">$C$57*POWER(10,-2)*E46-2.5*10</f>
-        <v>19.978999999999999</v>
+        <v>23.125499999999995</v>
       </c>
       <c r="G46" s="36">
         <f ca="1">AVERAGE(F46:F55)</f>
-        <v>21.589949999999995</v>
+        <v>21.475399999999997</v>
       </c>
       <c r="H46" s="37"/>
     </row>
@@ -1874,11 +1878,11 @@
       </c>
       <c r="E47" s="4">
         <f t="shared" ref="E47:E55" ca="1" si="0">IF($G$19="В30",RANDBETWEEN(3750,3950),IF($G$19="В25",RANDBETWEEN(3450,3650),IF($G$19="B30",RANDBETWEEN(3750,3950),IF($G$19="B25",RANDBETWEEN(3450,3650),RANDBETWEEN(3100,3350)))))</f>
-        <v>3165</v>
+        <v>3115</v>
       </c>
       <c r="F47" s="20">
         <f ca="1">$C$57*POWER(10,-2)*E47-2.5*10</f>
-        <v>20.892499999999998</v>
+        <v>20.167499999999997</v>
       </c>
       <c r="G47" s="38"/>
       <c r="H47" s="39"/>
@@ -1893,11 +1897,11 @@
       </c>
       <c r="E48" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3132</v>
+        <v>3234</v>
       </c>
       <c r="F48" s="20">
         <f ca="1">$C$57*POWER(10,-2)*E48-2.5*10</f>
-        <v>20.413999999999994</v>
+        <v>21.892999999999994</v>
       </c>
       <c r="G48" s="38"/>
       <c r="H48" s="39"/>
@@ -1912,11 +1916,11 @@
       </c>
       <c r="E49" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3297</v>
+        <v>3165</v>
       </c>
       <c r="F49" s="20">
         <f t="shared" ref="F49:F55" ca="1" si="1">$C$57*POWER(10,-2)*E49-2.5*10</f>
-        <v>22.8065</v>
+        <v>20.892499999999998</v>
       </c>
       <c r="G49" s="38"/>
       <c r="H49" s="39"/>
@@ -1931,11 +1935,11 @@
       </c>
       <c r="E50" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3180</v>
+        <v>3308</v>
       </c>
       <c r="F50" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>21.11</v>
+        <v>22.965999999999994</v>
       </c>
       <c r="G50" s="38"/>
       <c r="H50" s="39"/>
@@ -1950,11 +1954,11 @@
       </c>
       <c r="E51" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3343</v>
+        <v>3101</v>
       </c>
       <c r="F51" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>23.473499999999994</v>
+        <v>19.964499999999994</v>
       </c>
       <c r="G51" s="38"/>
       <c r="H51" s="39"/>
@@ -1969,11 +1973,11 @@
       </c>
       <c r="E52" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3244</v>
+        <v>3160</v>
       </c>
       <c r="F52" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>22.037999999999997</v>
+        <v>20.82</v>
       </c>
       <c r="G52" s="38"/>
       <c r="H52" s="39"/>
@@ -1988,11 +1992,11 @@
       </c>
       <c r="E53" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3202</v>
+        <v>3183</v>
       </c>
       <c r="F53" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>21.428999999999995</v>
+        <v>21.153499999999994</v>
       </c>
       <c r="G53" s="38"/>
       <c r="H53" s="39"/>
@@ -2007,11 +2011,11 @@
       </c>
       <c r="E54" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3321</v>
+        <v>3269</v>
       </c>
       <c r="F54" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>23.154499999999999</v>
+        <v>22.400499999999994</v>
       </c>
       <c r="G54" s="38"/>
       <c r="H54" s="39"/>
@@ -2026,11 +2030,11 @@
       </c>
       <c r="E55" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>3145</v>
+        <v>3198</v>
       </c>
       <c r="F55" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>20.602499999999999</v>
+        <v>21.370999999999995</v>
       </c>
       <c r="G55" s="40"/>
       <c r="H55" s="41"/>

</xml_diff>